<commit_message>
docs: Added new debts for HK Government
</commit_message>
<xml_diff>
--- a/Income And Expenses Forecast.xlsx
+++ b/Income And Expenses Forecast.xlsx
@@ -5802,7 +5802,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -7412,7 +7412,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B27")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -7528,7 +7528,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6880</v>
+        <v>-333029.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -8679,7 +8679,7 @@
       <c r="I193" s="40"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
@@ -9211,7 +9211,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -10821,7 +10821,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B30")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -10937,7 +10937,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -10953,7 +10953,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6880</v>
+        <v>-333029.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -12088,7 +12088,7 @@
       <c r="I193" s="40"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
@@ -12621,7 +12621,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -14231,7 +14231,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B33")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -14347,7 +14347,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6880</v>
+        <v>-333029.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -15498,7 +15498,7 @@
       <c r="I193" s="40"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
@@ -16030,7 +16030,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -17640,7 +17640,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B36")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -17756,7 +17756,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -17772,7 +17772,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6880</v>
+        <v>-333029.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -18907,7 +18907,7 @@
       <c r="I193" s="40"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
@@ -19440,7 +19440,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -21050,7 +21050,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B39")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -21166,7 +21166,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -21182,7 +21182,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6880</v>
+        <v>-333029.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -22317,7 +22317,7 @@
       <c r="I193" s="40"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
@@ -22849,7 +22849,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -24459,7 +24459,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B42")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -24575,7 +24575,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -24591,7 +24591,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6880</v>
+        <v>-333029.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -25727,7 +25727,7 @@
     </row>
     <row r="194" ht="24.75" customHeight="1"/>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
@@ -26258,7 +26258,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -27826,7 +27826,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B45")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -27942,7 +27942,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -27958,7 +27958,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -29560,7 +29560,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -31127,7 +31127,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B48")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -31243,7 +31243,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -31259,7 +31259,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -32863,7 +32863,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -34431,7 +34431,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B51")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -34547,7 +34547,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -34563,7 +34563,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -36590,7 +36590,7 @@
     <row r="133" s="238" customFormat="1" ht="20.25" customHeight="1"/>
     <row r="134" s="238" customFormat="1" ht="20.25" customHeight="1"/>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" objects="1"/>
+  <sheetProtection formatCells="0"/>
   <mergeCells count="19">
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A5:A6"/>
@@ -36714,7 +36714,7 @@
       </c>
       <c r="N3" s="211">
         <f>-C122</f>
-        <v>-24333</v>
+        <v>-350482.51</v>
       </c>
     </row>
     <row r="4" ht="35" customHeight="1" spans="1:14">
@@ -36746,7 +36746,7 @@
       </c>
       <c r="N4" s="211">
         <f ca="1">'July 2024 - September 2024'!C5</f>
-        <v>-11683</v>
+        <v>-337832.51</v>
       </c>
     </row>
     <row r="5" ht="35" customHeight="1" spans="1:14">
@@ -36778,7 +36778,7 @@
       </c>
       <c r="N5" s="211">
         <f ca="1">'October 2024 - December 2024'!C5</f>
-        <v>-10683</v>
+        <v>-336832.51</v>
       </c>
     </row>
     <row r="6" ht="35" customHeight="1" spans="1:14">
@@ -36810,7 +36810,7 @@
       </c>
       <c r="N6" s="211">
         <f ca="1">'January 2025 - March 2025'!C5</f>
-        <v>-6983</v>
+        <v>-333132.51</v>
       </c>
     </row>
     <row r="7" ht="35" customHeight="1" spans="1:14">
@@ -36842,7 +36842,7 @@
       </c>
       <c r="N7" s="211">
         <f ca="1">'April 2025 - June 2025'!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="8" ht="35" customHeight="1" spans="1:14">
@@ -36875,7 +36875,7 @@
       </c>
       <c r="N8" s="211">
         <f ca="1">'July 2025 - September 2025'!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="9" ht="35" customHeight="1" spans="1:14">
@@ -36907,7 +36907,7 @@
       </c>
       <c r="N9" s="221">
         <f ca="1">'October 2025 - December 2025'!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="10" ht="35" customHeight="1" spans="1:14">
@@ -36939,7 +36939,7 @@
       </c>
       <c r="N10" s="211">
         <f ca="1">'January 2026 - March 2026'!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="11" ht="35" customHeight="1" spans="1:14">
@@ -36972,7 +36972,7 @@
       </c>
       <c r="N11" s="215">
         <f ca="1">'April 2026 - June 2026'!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="12" ht="35" customHeight="1" spans="1:14">
@@ -37004,7 +37004,7 @@
       </c>
       <c r="N12" s="215">
         <f ca="1">'July 2026 - September 2026'!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="13" ht="35" customHeight="1" spans="1:14">
@@ -37036,7 +37036,7 @@
       </c>
       <c r="N13" s="215">
         <f ca="1">'October 2026 - December 2026'!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="14" ht="35" customHeight="1" spans="1:14">
@@ -37068,7 +37068,7 @@
       </c>
       <c r="N14" s="215">
         <f ca="1">'January 2027 - March 2027'!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="15" ht="35" customHeight="1" spans="1:14">
@@ -37100,7 +37100,7 @@
       </c>
       <c r="N15" s="215">
         <f ca="1">'April 2027 - June 2027'!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="16" ht="35" customHeight="1" spans="1:14">
@@ -37134,7 +37134,7 @@
       </c>
       <c r="N16" s="215">
         <f ca="1">Forecast_14!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="17" ht="35" customHeight="1" spans="9:14">
@@ -37152,7 +37152,7 @@
       </c>
       <c r="N17" s="215">
         <f ca="1">Forecast_15!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="18" ht="35" customHeight="1" spans="9:14">
@@ -37170,7 +37170,7 @@
       </c>
       <c r="N18" s="211">
         <f ca="1">Forecast_16!C5</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
     </row>
     <row r="19" ht="35" customHeight="1" spans="9:10">
@@ -38338,7 +38338,7 @@
       </c>
       <c r="B116" s="199"/>
       <c r="C116" s="234">
-        <v>0</v>
+        <v>326149.51</v>
       </c>
       <c r="D116" s="14"/>
       <c r="E116" s="14"/>
@@ -38415,7 +38415,7 @@
       </c>
       <c r="C122" s="223">
         <f>SUM(C112:C121)</f>
-        <v>24333</v>
+        <v>350482.51</v>
       </c>
     </row>
     <row r="123" ht="35" customHeight="1" spans="1:3">
@@ -38425,7 +38425,7 @@
       </c>
       <c r="C123" s="36">
         <f>C122+C110</f>
-        <v>25836</v>
+        <v>351985.51</v>
       </c>
     </row>
     <row r="124" ht="35" customHeight="1" spans="5:5">
@@ -39764,7 +39764,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-11683</v>
+        <v>-337832.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -41406,7 +41406,7 @@
       </c>
       <c r="C102" s="108" cm="1">
         <f ca="1" t="array" ref="C102">(((INDIRECT("'"&amp;INDIRECT("Main!B9")&amp;"'!E135")+INDIRECT("'"&amp;INDIRECT("Main!B9")&amp;"'!E162")+INDIRECT("'"&amp;INDIRECT("Main!B9")&amp;"'!E189")))+SUM(E122+E149+E176))-INDIRECT("'"&amp;INDIRECT("Main!B9")&amp;"'!C116")</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="164"/>
@@ -41522,7 +41522,7 @@
       </c>
       <c r="C108" s="108">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-11683</v>
+        <v>-337832.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -41538,7 +41538,7 @@
       </c>
       <c r="C109" s="108">
         <f ca="1">C108-C96</f>
-        <v>-13711.5</v>
+        <v>-339861.01</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -43214,7 +43214,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-10683</v>
+        <v>-336832.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -44886,7 +44886,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B12")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -45002,7 +45002,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-10683</v>
+        <v>-336832.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -45018,7 +45018,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-12052</v>
+        <v>-338201.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -46764,7 +46764,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6983</v>
+        <v>-333132.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -48420,7 +48420,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B15")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -48536,7 +48536,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6983</v>
+        <v>-333132.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -48552,7 +48552,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-7380</v>
+        <v>-333529.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -49705,7 +49705,7 @@
       <c r="I193" s="40"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
@@ -50282,7 +50282,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -51896,7 +51896,7 @@
       </c>
       <c r="C102" s="36" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B18")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -52012,7 +52012,7 @@
       </c>
       <c r="C108" s="36">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -52028,7 +52028,7 @@
       </c>
       <c r="C109" s="36">
         <f ca="1">C108-C96</f>
-        <v>-6880</v>
+        <v>-333029.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -53169,7 +53169,7 @@
       <c r="I193" s="40"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
@@ -53729,7 +53729,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -55339,7 +55339,7 @@
       </c>
       <c r="C102" s="108" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B21")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -55455,7 +55455,7 @@
       </c>
       <c r="C108" s="108">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -55471,7 +55471,7 @@
       </c>
       <c r="C109" s="108">
         <f ca="1">C108-C96</f>
-        <v>-6880</v>
+        <v>-333029.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -56612,7 +56612,7 @@
       <c r="I193" s="40"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>
@@ -57167,7 +57167,7 @@
       <c r="B5" s="11"/>
       <c r="C5" s="12">
         <f ca="1">C108</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -58773,7 +58773,7 @@
       </c>
       <c r="C102" s="108" cm="1">
         <f ca="1" t="array" ref="C102">INDIRECT("'"&amp;INDIRECT("Main!B24")&amp;"'!C102")+SUM(E122+E149+E176)</f>
-        <v>0</v>
+        <v>-326149.51</v>
       </c>
       <c r="D102" s="14"/>
       <c r="E102" s="14"/>
@@ -58889,7 +58889,7 @@
       </c>
       <c r="C108" s="108">
         <f ca="1">SUM(C98:C107)</f>
-        <v>-6483</v>
+        <v>-332632.51</v>
       </c>
       <c r="D108" s="14"/>
       <c r="E108" s="14"/>
@@ -58905,7 +58905,7 @@
       </c>
       <c r="C109" s="108">
         <f ca="1">C108-C96</f>
-        <v>-6880</v>
+        <v>-333029.51</v>
       </c>
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
@@ -60040,7 +60040,7 @@
       <c r="I193" s="40"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" objects="1"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="174">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C2:G2"/>

</xml_diff>

<commit_message>
docs: 1. Updated Expenses 2. Top up value for Google Play.
</commit_message>
<xml_diff>
--- a/Income And Expenses Forecast.xlsx
+++ b/Income And Expenses Forecast.xlsx
@@ -1218,10 +1218,12 @@
     <t>Birdie Paid in advance</t>
   </si>
   <si>
-    <t>1.  yuu</t>
+    <t>1.  yuu
+2. Google Play</t>
   </si>
   <si>
-    <t>1. Newly added / remain yuu points ~ $1</t>
+    <t>1. Newly added / remain yuu points ~ $1
+2. Google Play Newly top up $136</t>
   </si>
   <si>
     <t>31th May 2025</t>
@@ -5745,7 +5747,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -5761,7 +5763,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>4648.7</v>
+        <v>4784.7</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -5777,7 +5779,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>5694.2</v>
+        <v>5966.2</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -7629,7 +7631,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B27")&amp;"'!E190")</f>
-        <v>2571.6</v>
+        <v>2707.6</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -7901,7 +7903,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>3414.3</v>
+        <v>3550.3</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -7993,7 +7995,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>3414.3</v>
+        <v>3550.3</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -8265,7 +8267,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>3806</v>
+        <v>3942</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -8357,7 +8359,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>3806</v>
+        <v>3942</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -8629,7 +8631,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>4648.7</v>
+        <v>4784.7</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -9154,7 +9156,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -9170,7 +9172,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>6434.8</v>
+        <v>6570.8</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -9186,7 +9188,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>7480.3</v>
+        <v>7752.3</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -11038,7 +11040,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B30")&amp;"'!E190")</f>
-        <v>4648.7</v>
+        <v>4784.7</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -11310,7 +11312,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>5200.4</v>
+        <v>5336.4</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -11402,7 +11404,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>5200.4</v>
+        <v>5336.4</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -11674,7 +11676,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>5883.1</v>
+        <v>6019.1</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -11766,7 +11768,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>5883.1</v>
+        <v>6019.1</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -12038,7 +12040,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>6434.8</v>
+        <v>6570.8</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -12564,7 +12566,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -12580,7 +12582,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>8449</v>
+        <v>8585</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -12596,7 +12598,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>9494.5</v>
+        <v>9766.5</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -14448,7 +14450,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B33")&amp;"'!E190")</f>
-        <v>6434.8</v>
+        <v>6570.8</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -14720,7 +14722,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>7277.5</v>
+        <v>7413.5</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -14812,7 +14814,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>7277.5</v>
+        <v>7413.5</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -15084,7 +15086,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>7669.2</v>
+        <v>7805.2</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -15176,7 +15178,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>7669.2</v>
+        <v>7805.2</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -15448,7 +15450,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>8449</v>
+        <v>8585</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -15973,7 +15975,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -15989,7 +15991,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>10235.1</v>
+        <v>10371.1</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -16005,7 +16007,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>11280.6</v>
+        <v>11552.6</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -17857,7 +17859,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B36")&amp;"'!E190")</f>
-        <v>8449</v>
+        <v>8585</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -18129,7 +18131,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>9000.7</v>
+        <v>9136.7</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -18221,7 +18223,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>9000.7</v>
+        <v>9136.7</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -18493,7 +18495,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>9683.4</v>
+        <v>9819.4</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -18585,7 +18587,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>9683.4</v>
+        <v>9819.4</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -18857,7 +18859,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>10235.1</v>
+        <v>10371.1</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -19383,7 +19385,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -19399,7 +19401,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>12312.2</v>
+        <v>12448.2</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -19415,7 +19417,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>13357.7</v>
+        <v>13629.7</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -21267,7 +21269,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B39")&amp;"'!E190")</f>
-        <v>10235.1</v>
+        <v>10371.1</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -21539,7 +21541,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>11077.8</v>
+        <v>11213.8</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -21631,7 +21633,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>11077.8</v>
+        <v>11213.8</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -21903,7 +21905,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>11469.5</v>
+        <v>11605.5</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -21995,7 +21997,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>11469.5</v>
+        <v>11605.5</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -22267,7 +22269,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>12312.2</v>
+        <v>12448.2</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -22792,7 +22794,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -22808,7 +22810,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -22824,7 +22826,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>15143.8</v>
+        <v>15415.8</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -24676,7 +24678,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B42")&amp;"'!E190")</f>
-        <v>12312.2</v>
+        <v>12448.2</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -24948,7 +24950,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>12863.9</v>
+        <v>12999.9</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -25040,7 +25042,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>12863.9</v>
+        <v>12999.9</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -25312,7 +25314,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>13546.6</v>
+        <v>13682.6</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -25404,7 +25406,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>13546.6</v>
+        <v>13682.6</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -25676,7 +25678,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -26201,7 +26203,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -26217,7 +26219,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -26233,7 +26235,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>15143.8</v>
+        <v>15415.8</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -28043,7 +28045,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B45")&amp;"'!E190")</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -28311,7 +28313,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -28403,7 +28405,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -28671,7 +28673,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -28763,7 +28765,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -29031,7 +29033,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -29503,7 +29505,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -29519,7 +29521,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -29535,7 +29537,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>15143.8</v>
+        <v>15415.8</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -31344,7 +31346,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B48")&amp;"'!E190")</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -31612,7 +31614,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -31704,7 +31706,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -31972,7 +31974,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -32064,7 +32066,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -32332,7 +32334,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -32806,7 +32808,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -32822,7 +32824,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -32838,7 +32840,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>15143.8</v>
+        <v>15415.8</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -34648,7 +34650,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B51")&amp;"'!E190")</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -34916,7 +34918,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -35008,7 +35010,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -35276,7 +35278,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -35368,7 +35370,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -35636,7 +35638,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -36689,7 +36691,7 @@
         <v>34</v>
       </c>
       <c r="F3" s="197">
-        <v>1072.1</v>
+        <v>875.3</v>
       </c>
       <c r="I3" s="205" t="str">
         <f>TEXT(Main!B3,"dd mmmm yyyy")&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,1)-1,"dd mmmm yyyy"),TEXT(Main!B3+(Main!B5-Main!B3)*1,"dd mmmm yyyy"))</f>
@@ -36817,7 +36819,7 @@
         <v>38</v>
       </c>
       <c r="F7" s="197">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="I7" s="208" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,4),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*4)+4,"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,5)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*5+4),"dd mmmm yyyy"))</f>
@@ -36972,7 +36974,7 @@
         <v>43</v>
       </c>
       <c r="C12" s="169">
-        <v>2</v>
+        <v>138</v>
       </c>
       <c r="D12" s="171"/>
       <c r="E12" s="199" t="s">
@@ -37011,7 +37013,7 @@
         <v>44</v>
       </c>
       <c r="F13" s="197">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I13" s="209" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,10),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*10)+10,"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,11)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*11+10),"dd mmmm yyyy"))</f>
@@ -37083,7 +37085,7 @@
       </c>
       <c r="J15" s="210">
         <f ca="1">'April 2025 - June 2025'!E136</f>
-        <v>920.500000000001</v>
+        <v>1056.5</v>
       </c>
       <c r="M15" s="207" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,36),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*36+36),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,39)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*39+38),"dd mmmm yyyy"))</f>
@@ -37101,7 +37103,7 @@
       </c>
       <c r="C16" s="175">
         <f>SUM(C3:C15)</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D16" s="176"/>
       <c r="E16" s="174" t="s">
@@ -37109,7 +37111,7 @@
       </c>
       <c r="F16" s="200">
         <f>SUM(F3:F15)</f>
-        <v>1252.5</v>
+        <v>1045.5</v>
       </c>
       <c r="I16" s="211" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,13),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*13)+13,"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,14)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*14+13),"dd mmmm yyyy"))</f>
@@ -37117,7 +37119,7 @@
       </c>
       <c r="J16" s="210">
         <f ca="1">'April 2025 - June 2025'!E163</f>
-        <v>1071.5</v>
+        <v>1207.5</v>
       </c>
       <c r="M16" s="207" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,39),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*39+39),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,42)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*42+41),"dd mmmm yyyy"))</f>
@@ -37135,7 +37137,7 @@
       </c>
       <c r="J17" s="210">
         <f ca="1">'April 2025 - June 2025'!E190</f>
-        <v>831.500000000001</v>
+        <v>967.500000000001</v>
       </c>
       <c r="M17" s="207" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,42),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*42+42),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,45)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*45+44),"dd mmmm yyyy"))</f>
@@ -37153,7 +37155,7 @@
       </c>
       <c r="J18" s="210">
         <f ca="1">'July 2025 - September 2025'!E136</f>
-        <v>697.500000000001</v>
+        <v>833.500000000001</v>
       </c>
       <c r="M18" s="207" t="str">
         <f>IF(Main!B2,TEXT(EDATE(Main!B3,45),"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*45+45),"dd mmmm yyyy"))&amp;" - "&amp;IF(Main!B2,TEXT(EDATE(Main!B3,48)-1,"dd mmmm yyyy"),TEXT(Main!B3+((Main!B5-Main!B3)*48+47),"dd mmmm yyyy"))</f>
@@ -37171,7 +37173,7 @@
       </c>
       <c r="J19" s="210">
         <f ca="1">'July 2025 - September 2025'!E163</f>
-        <v>707.500000000001</v>
+        <v>843.500000000001</v>
       </c>
     </row>
     <row r="20" ht="35" customHeight="1" spans="9:10">
@@ -37181,7 +37183,7 @@
       </c>
       <c r="J20" s="210">
         <f ca="1">'July 2025 - September 2025'!E190</f>
-        <v>639.500000000001</v>
+        <v>775.500000000001</v>
       </c>
     </row>
     <row r="21" ht="35" customHeight="1" spans="9:10">
@@ -37191,7 +37193,7 @@
       </c>
       <c r="J21" s="210">
         <f ca="1">'October 2025 - December 2025'!E136</f>
-        <v>1227.2</v>
+        <v>1363.2</v>
       </c>
     </row>
     <row r="22" ht="35" customHeight="1" spans="1:10">
@@ -37211,7 +37213,7 @@
       </c>
       <c r="J22" s="210">
         <f ca="1">'October 2025 - December 2025'!E163</f>
-        <v>2019.9</v>
+        <v>2155.9</v>
       </c>
     </row>
     <row r="23" ht="35" customHeight="1" spans="1:10">
@@ -37236,7 +37238,7 @@
       </c>
       <c r="J23" s="210">
         <f ca="1">'October 2025 - December 2025'!E190</f>
-        <v>2571.6</v>
+        <v>2707.6</v>
       </c>
     </row>
     <row r="24" ht="35" customHeight="1" spans="1:10">
@@ -37261,7 +37263,7 @@
       </c>
       <c r="J24" s="210">
         <f ca="1">'January 2026 - March 2026'!E136</f>
-        <v>3414.3</v>
+        <v>3550.3</v>
       </c>
     </row>
     <row r="25" ht="35" customHeight="1" spans="1:10">
@@ -37280,7 +37282,7 @@
       </c>
       <c r="J25" s="210">
         <f ca="1">'January 2026 - March 2026'!E163</f>
-        <v>3806</v>
+        <v>3942</v>
       </c>
     </row>
     <row r="26" ht="35" customHeight="1" spans="1:10">
@@ -37299,7 +37301,7 @@
       </c>
       <c r="J26" s="210">
         <f ca="1">'January 2026 - March 2026'!E190</f>
-        <v>4648.7</v>
+        <v>4784.7</v>
       </c>
     </row>
     <row r="27" ht="35" customHeight="1" spans="1:10">
@@ -37318,7 +37320,7 @@
       </c>
       <c r="J27" s="210">
         <f ca="1">'April 2026 - June 2026'!E136</f>
-        <v>5200.4</v>
+        <v>5336.4</v>
       </c>
     </row>
     <row r="28" ht="35" customHeight="1" spans="1:10">
@@ -37337,7 +37339,7 @@
       </c>
       <c r="J28" s="210">
         <f ca="1">'April 2026 - June 2026'!E163</f>
-        <v>5883.1</v>
+        <v>6019.1</v>
       </c>
     </row>
     <row r="29" ht="35" customHeight="1" spans="1:10">
@@ -37356,7 +37358,7 @@
       </c>
       <c r="J29" s="206">
         <f ca="1">'April 2026 - June 2026'!E190</f>
-        <v>6434.8</v>
+        <v>6570.8</v>
       </c>
     </row>
     <row r="30" ht="35" customHeight="1" spans="1:10">
@@ -37378,7 +37380,7 @@
       </c>
       <c r="J30" s="214">
         <f ca="1">'July 2026 - September 2026'!E136</f>
-        <v>7277.5</v>
+        <v>7413.5</v>
       </c>
     </row>
     <row r="31" ht="35" customHeight="1" spans="9:10">
@@ -37388,7 +37390,7 @@
       </c>
       <c r="J31" s="210">
         <f ca="1">'July 2026 - September 2026'!E163</f>
-        <v>7669.2</v>
+        <v>7805.2</v>
       </c>
     </row>
     <row r="32" ht="35" customHeight="1" spans="9:10">
@@ -37398,7 +37400,7 @@
       </c>
       <c r="J32" s="210">
         <f ca="1">'July 2026 - September 2026'!E190</f>
-        <v>8449</v>
+        <v>8585</v>
       </c>
     </row>
     <row r="33" ht="35" customHeight="1" spans="9:10">
@@ -37408,7 +37410,7 @@
       </c>
       <c r="J33" s="210">
         <f ca="1">'October 2026 - December 2026'!E136</f>
-        <v>9000.7</v>
+        <v>9136.7</v>
       </c>
     </row>
     <row r="34" ht="35" customHeight="1" spans="1:10">
@@ -37428,7 +37430,7 @@
       </c>
       <c r="J34" s="210">
         <f ca="1">'October 2026 - December 2026'!E163</f>
-        <v>9683.4</v>
+        <v>9819.4</v>
       </c>
     </row>
     <row r="35" ht="35" customHeight="1" spans="1:10">
@@ -37453,7 +37455,7 @@
       </c>
       <c r="J35" s="210">
         <f ca="1">'October 2026 - December 2026'!E190</f>
-        <v>10235.1</v>
+        <v>10371.1</v>
       </c>
     </row>
     <row r="36" ht="35" customHeight="1" spans="1:10">
@@ -37478,7 +37480,7 @@
       </c>
       <c r="J36" s="210">
         <f ca="1">'January 2027 - March 2027'!E136</f>
-        <v>11077.8</v>
+        <v>11213.8</v>
       </c>
     </row>
     <row r="37" ht="35" customHeight="1" spans="1:10">
@@ -37503,7 +37505,7 @@
       </c>
       <c r="J37" s="210">
         <f ca="1">'January 2027 - March 2027'!E163</f>
-        <v>11469.5</v>
+        <v>11605.5</v>
       </c>
     </row>
     <row r="38" ht="35" customHeight="1" spans="1:10">
@@ -37528,7 +37530,7 @@
       </c>
       <c r="J38" s="210">
         <f ca="1">'January 2027 - March 2027'!E190</f>
-        <v>12312.2</v>
+        <v>12448.2</v>
       </c>
     </row>
     <row r="39" ht="35" customHeight="1" spans="1:10">
@@ -37547,7 +37549,7 @@
       </c>
       <c r="J39" s="210">
         <f ca="1">'April 2027 - June 2027'!E136</f>
-        <v>12863.9</v>
+        <v>12999.9</v>
       </c>
     </row>
     <row r="40" ht="35" customHeight="1" spans="1:10">
@@ -37566,7 +37568,7 @@
       </c>
       <c r="J40" s="210">
         <f ca="1">'April 2027 - June 2027'!E163</f>
-        <v>13546.6</v>
+        <v>13682.6</v>
       </c>
     </row>
     <row r="41" ht="35" customHeight="1" spans="1:10">
@@ -37585,7 +37587,7 @@
       </c>
       <c r="J41" s="210">
         <f ca="1">'April 2027 - June 2027'!E190</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="42" ht="35" customHeight="1" spans="1:10">
@@ -37607,7 +37609,7 @@
       </c>
       <c r="J42" s="210">
         <f ca="1">Forecast_14!E136</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="43" ht="35" customHeight="1" spans="9:10">
@@ -37617,7 +37619,7 @@
       </c>
       <c r="J43" s="210">
         <f ca="1">Forecast_14!E163</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="44" ht="35" customHeight="1" spans="9:10">
@@ -37627,7 +37629,7 @@
       </c>
       <c r="J44" s="210">
         <f ca="1">Forecast_14!E190</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="45" ht="35" customHeight="1" spans="9:10">
@@ -37637,7 +37639,7 @@
       </c>
       <c r="J45" s="210">
         <f ca="1">Forecast_15!E136</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="46" ht="35" customHeight="1" spans="1:10">
@@ -37657,7 +37659,7 @@
       </c>
       <c r="J46" s="210">
         <f ca="1">Forecast_15!E163</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="47" ht="35" customHeight="1" spans="1:10">
@@ -37682,7 +37684,7 @@
       </c>
       <c r="J47" s="210">
         <f ca="1">Forecast_15!E190</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="48" ht="35" customHeight="1" spans="1:10">
@@ -37707,7 +37709,7 @@
       </c>
       <c r="J48" s="210">
         <f ca="1">Forecast_16!E136</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="49" ht="35" customHeight="1" spans="1:10">
@@ -37732,7 +37734,7 @@
       </c>
       <c r="J49" s="210">
         <f ca="1">Forecast_16!E163</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="50" ht="35" customHeight="1" spans="1:10">
@@ -37757,7 +37759,7 @@
       </c>
       <c r="J50" s="206">
         <f ca="1">Forecast_16!E190</f>
-        <v>14098.3</v>
+        <v>14234.3</v>
       </c>
     </row>
     <row r="51" ht="35" customHeight="1" spans="1:7">
@@ -39711,7 +39713,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -39739,7 +39741,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>1548.21</v>
+        <v>1684.21</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -43161,7 +43163,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -43189,7 +43191,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>1218.84</v>
+        <v>1354.84</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -46707,7 +46709,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -46739,7 +46741,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>1212</v>
+        <v>1348</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -50225,7 +50227,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -50241,7 +50243,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>831.500000000001</v>
+        <v>967.500000000001</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -50257,7 +50259,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>1877</v>
+        <v>2149</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -50407,7 +50409,7 @@
       <c r="H13" s="14"/>
       <c r="I13" s="47"/>
     </row>
-    <row r="14" ht="20" customHeight="1" spans="1:9">
+    <row r="14" ht="49" customHeight="1" spans="1:9">
       <c r="A14" s="19"/>
       <c r="B14" s="110" t="s">
         <v>255</v>
@@ -50418,7 +50420,7 @@
       </c>
       <c r="E14" s="111"/>
       <c r="F14" s="41">
-        <v>1</v>
+        <v>137</v>
       </c>
       <c r="G14" s="42"/>
       <c r="H14" s="14"/>
@@ -50447,7 +50449,7 @@
       <c r="E16" s="44"/>
       <c r="F16" s="45">
         <f>SUM(F10:G15)</f>
-        <v>2486</v>
+        <v>2622</v>
       </c>
       <c r="G16" s="46"/>
       <c r="H16" s="14"/>
@@ -52391,7 +52393,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>920.500000000001</v>
+        <v>1056.5</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -52483,7 +52485,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>920.500000000001</v>
+        <v>1056.5</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -52757,7 +52759,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>1071.5</v>
+        <v>1207.5</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -52849,7 +52851,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>1071.5</v>
+        <v>1207.5</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -53123,7 +53125,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>831.500000000001</v>
+        <v>967.500000000001</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -53676,7 +53678,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -53692,7 +53694,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>639.500000000001</v>
+        <v>775.500000000001</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -53708,7 +53710,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>1685</v>
+        <v>1957</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -55562,7 +55564,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B21")&amp;"'!E190")</f>
-        <v>831.500000000001</v>
+        <v>967.500000000001</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -55836,7 +55838,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>697.500000000001</v>
+        <v>833.500000000001</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -55928,7 +55930,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>697.500000000001</v>
+        <v>833.500000000001</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -56202,7 +56204,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>707.500000000001</v>
+        <v>843.500000000001</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -56294,7 +56296,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>707.500000000001</v>
+        <v>843.500000000001</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -56570,7 +56572,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>639.500000000001</v>
+        <v>775.500000000001</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>
@@ -57123,7 +57125,7 @@
       </c>
       <c r="C2" s="4" cm="1">
         <f ca="1" t="array" ref="C2">INDIRECT("'"&amp;Main!B9&amp;"'!$C$16")</f>
-        <v>1045.5</v>
+        <v>1181.5</v>
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -57139,7 +57141,7 @@
       </c>
       <c r="C3" s="7">
         <f ca="1">E190</f>
-        <v>2571.6</v>
+        <v>2707.6</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -57155,7 +57157,7 @@
       <c r="B4" s="9"/>
       <c r="C4" s="10">
         <f ca="1">SUM(C2:G3)</f>
-        <v>3617.1</v>
+        <v>3889.1</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
@@ -59003,7 +59005,7 @@
       <c r="D116" s="57"/>
       <c r="E116" s="70" cm="1">
         <f ca="1" t="array" ref="E116">INDIRECT("'"&amp;INDIRECT("Main!B24")&amp;"'!E190")</f>
-        <v>639.500000000001</v>
+        <v>775.500000000001</v>
       </c>
       <c r="F116" s="14"/>
       <c r="G116" s="14"/>
@@ -59277,7 +59279,7 @@
       <c r="D136" s="81"/>
       <c r="E136" s="87">
         <f ca="1">(F16+E116)-(SUM(E118:E127)+SUM(E129:E135))</f>
-        <v>1227.2</v>
+        <v>1363.2</v>
       </c>
       <c r="F136" s="14"/>
       <c r="G136" s="14"/>
@@ -59369,7 +59371,7 @@
       <c r="D143" s="57"/>
       <c r="E143" s="87">
         <f ca="1">E136</f>
-        <v>1227.2</v>
+        <v>1363.2</v>
       </c>
       <c r="F143" s="14"/>
       <c r="G143" s="14"/>
@@ -59641,7 +59643,7 @@
       <c r="D163" s="81"/>
       <c r="E163" s="90">
         <f ca="1">(F28+E143)-(SUM(E145:E154)+SUM(E156:E162))</f>
-        <v>2019.9</v>
+        <v>2155.9</v>
       </c>
       <c r="F163" s="14"/>
       <c r="G163" s="14"/>
@@ -59733,7 +59735,7 @@
       <c r="D170" s="57"/>
       <c r="E170" s="90">
         <f ca="1">E163</f>
-        <v>2019.9</v>
+        <v>2155.9</v>
       </c>
       <c r="F170" s="14"/>
       <c r="G170" s="14"/>
@@ -60005,7 +60007,7 @@
       <c r="D190" s="81"/>
       <c r="E190" s="90">
         <f ca="1">(F40+E170)-(SUM(E172:E181)+SUM(E183:E189))</f>
-        <v>2571.6</v>
+        <v>2707.6</v>
       </c>
       <c r="F190" s="14"/>
       <c r="G190" s="14"/>

</xml_diff>